<commit_message>
feat(finance): add Margin Calculator (CVP) tab to RIVR Tech forecast
New 'Margin Calculator' tab answers 'what revenue do we need for an X%
profit' using cost-volume-profit math on pre-tax operating profit:
  Required revenue = FixedCosts / (1 - variableCost% - targetMargin)

- Editable (placeholder) cost structure: variable % of revenue + itemized
  fixed costs; contribution margin, breakeven, margin of safety.
- Target solver by margin % and by profit $; 0-30% sensitivity table with
  feasibility flags; operating margin at each scenario's revenue.
- Links revenue from Consolidated (active scenario) with optional override.
- Data Dictionary extended with CVP terms; README documents the tab with a
  worked example (10% margin => $13.85M required revenue).
- Validated: 0 formula errors across 2,515 formulas; cached values embedded.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018n21dnmsv1yZa9nLHfN5ph
</commit_message>
<xml_diff>
--- a/RIVR_Tech_2027_Revenue_Forecast.xlsx
+++ b/RIVR_Tech_2027_Revenue_Forecast.xlsx
@@ -15,7 +15,8 @@
     <sheet name="Consolidated Revenue" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Scenario Analysis" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Annual Summary" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Data Dictionary" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Margin Calculator" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Data Dictionary" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Key Assumptions'!$A$65:$T$90</definedName>
@@ -34,7 +35,7 @@
     <numFmt numFmtId="168" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="169" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -108,6 +109,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00006100"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00C00000"/>
       <sz val="9"/>
     </font>
     <font>
@@ -272,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -281,26 +288,26 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -456,6 +463,38 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -469,7 +508,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="11">
     <dxf>
       <font>
         <b val="1"/>
@@ -521,6 +560,46 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="009C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="00006100"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="009C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
         <color rgb="009C0006"/>
       </font>
     </dxf>
@@ -1241,6 +1320,36 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>RIVR Model</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Costs that scale with revenue: bandwidth/IP transit, transport, payment processing, sales commissions, variable support. PLACEHOLDER.</t>
+      </text>
+    </comment>
+    <comment ref="B17" authorId="0" shapeId="0">
+      <text>
+        <t>Leave blank to use the forecast. Enter a number to test any revenue level.</t>
+      </text>
+    </comment>
+    <comment ref="B29" authorId="0" shapeId="0">
+      <text>
+        <t>Enter the profit margin you want (e.g. 10%). The calculator returns the revenue needed to achieve it at the current cost structure.</t>
+      </text>
+    </comment>
+    <comment ref="B36" authorId="0" shapeId="0">
+      <text>
+        <t>Alternatively, enter a target profit in dollars. Returns the revenue needed to hit that profit.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -2059,6 +2168,503 @@
 </s:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00808080"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DATA DICTIONARY &amp; DEFINITIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Definitions of every major term, assumption, and calculation used in this workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="47" t="inlineStr">
+        <is>
+          <t>Term / Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="47" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="C3" s="47" t="inlineStr">
+        <is>
+          <t>Where used / Formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="99" t="inlineStr">
+        <is>
+          <t>ARPU</t>
+        </is>
+      </c>
+      <c r="B4" s="100" t="inlineStr">
+        <is>
+          <t>Average Revenue Per User — recurring revenue divided by the average number of billable customers in a month.</t>
+        </is>
+      </c>
+      <c r="C4" s="101" t="inlineStr">
+        <is>
+          <t>Recurring revenue / Avg billable subs</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="99" t="inlineStr">
+        <is>
+          <t>MRR</t>
+        </is>
+      </c>
+      <c r="B5" s="100" t="inlineStr">
+        <is>
+          <t>Monthly Recurring Revenue — contractually recurring revenue in a month, excluding one-time charges (installation, activation, construction, upfront IRU).</t>
+        </is>
+      </c>
+      <c r="C5" s="101" t="inlineStr">
+        <is>
+          <t>Total recurring revenue (Consolidated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="99" t="inlineStr">
+        <is>
+          <t>ARR run rate</t>
+        </is>
+      </c>
+      <c r="B6" s="100" t="inlineStr">
+        <is>
+          <t>Annualized Recurring Revenue — the current month's MRR multiplied by 12; a forward run-rate, not a sum of the year.</t>
+        </is>
+      </c>
+      <c r="C6" s="101" t="inlineStr">
+        <is>
+          <t>MRR x 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="99" t="inlineStr">
+        <is>
+          <t>Gross additions</t>
+        </is>
+      </c>
+      <c r="B7" s="100" t="inlineStr">
+        <is>
+          <t>New customers connected in a month before subtracting churn or disconnects.</t>
+        </is>
+      </c>
+      <c r="C7" s="101" t="inlineStr">
+        <is>
+          <t>Assumption × scenario add multiplier</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="99" t="inlineStr">
+        <is>
+          <t>Net additions</t>
+        </is>
+      </c>
+      <c r="B8" s="100" t="inlineStr">
+        <is>
+          <t>Gross additions + reconnects − churn disconnects − other disconnects.</t>
+        </is>
+      </c>
+      <c r="C8" s="101" t="inlineStr">
+        <is>
+          <t>Roll-forward</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="99" t="inlineStr">
+        <is>
+          <t>Churn</t>
+        </is>
+      </c>
+      <c r="B9" s="100" t="inlineStr">
+        <is>
+          <t>Customers who disconnect voluntarily or involuntarily. Monthly churn % is applied to the beginning subscriber base.</t>
+        </is>
+      </c>
+      <c r="C9" s="101" t="inlineStr">
+        <is>
+          <t>Beginning subs × churn % × churn multiplier</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="99" t="inlineStr">
+        <is>
+          <t>Reconnects</t>
+        </is>
+      </c>
+      <c r="B10" s="100" t="inlineStr">
+        <is>
+          <t>Previously disconnected customers who reconnect in the month; added back to the base.</t>
+        </is>
+      </c>
+      <c r="C10" s="101" t="inlineStr">
+        <is>
+          <t>Assumption input</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="99" t="inlineStr">
+        <is>
+          <t>Average billable customers</t>
+        </is>
+      </c>
+      <c r="B11" s="100" t="inlineStr">
+        <is>
+          <t>Convention for revenue timing. 'Average' = (beginning + ending)/2; alternatives are Beginning or Ending.</t>
+        </is>
+      </c>
+      <c r="C11" s="101" t="inlineStr">
+        <is>
+          <t>Key Assumptions convention cell</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="99" t="inlineStr">
+        <is>
+          <t>Recurring revenue</t>
+        </is>
+      </c>
+      <c r="B12" s="100" t="inlineStr">
+        <is>
+          <t>Revenue that repeats every month under a subscription or contract (broadband, DIA, static IP, managed Wi-Fi, dark fiber lease, O&amp;M).</t>
+        </is>
+      </c>
+      <c r="C12" s="101" t="inlineStr">
+        <is>
+          <t>Segment recurring rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="38" customHeight="1">
+      <c r="A13" s="99" t="inlineStr">
+        <is>
+          <t>One-time revenue</t>
+        </is>
+      </c>
+      <c r="B13" s="100" t="inlineStr">
+        <is>
+          <t>Non-repeating charges: installation, activation, aid-to-construction, professional services, upfront IRU proceeds.</t>
+        </is>
+      </c>
+      <c r="C13" s="101" t="inlineStr">
+        <is>
+          <t>Segment one-time rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="38" customHeight="1">
+      <c r="A14" s="99" t="inlineStr">
+        <is>
+          <t>IRU</t>
+        </is>
+      </c>
+      <c r="B14" s="100" t="inlineStr">
+        <is>
+          <t>Indefeasible Right of Use — a long-term (often 15-20 yr) prepaid right to use specific fiber strands. Upfront proceeds may be recognized immediately, straight-line over the term, or per a manual schedule. TREATMENT REQUIRES CFO / EXTERNAL ACCOUNTANT REVIEW UNDER ASC 606.</t>
+        </is>
+      </c>
+      <c r="C14" s="101" t="inlineStr">
+        <is>
+          <t>Dark Fiber Forecast IRU rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1">
+      <c r="A15" s="99" t="inlineStr">
+        <is>
+          <t>Dark fiber</t>
+        </is>
+      </c>
+      <c r="B15" s="100" t="inlineStr">
+        <is>
+          <t>Unlit optical fiber leased to a customer who provides their own optronics; billed as a monthly lease, strand/pair lease, or IRU.</t>
+        </is>
+      </c>
+      <c r="C15" s="101" t="inlineStr">
+        <is>
+          <t>Dark Fiber Forecast</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="A16" s="99" t="inlineStr">
+        <is>
+          <t>O&amp;M revenue</t>
+        </is>
+      </c>
+      <c r="B16" s="100" t="inlineStr">
+        <is>
+          <t>Operations &amp; Maintenance revenue — recurring fees for maintaining leased fiber (locates, splice repair, monitoring).</t>
+        </is>
+      </c>
+      <c r="C16" s="101" t="inlineStr">
+        <is>
+          <t>Dark Fiber Forecast O&amp;M row</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="38" customHeight="1">
+      <c r="A17" s="99" t="inlineStr">
+        <is>
+          <t>Revenue run rate</t>
+        </is>
+      </c>
+      <c r="B17" s="100" t="inlineStr">
+        <is>
+          <t>A forward-looking annualized figure derived from a single period (e.g., December MRR × 12).</t>
+        </is>
+      </c>
+      <c r="C17" s="101" t="inlineStr">
+        <is>
+          <t>ARR run rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="38" customHeight="1">
+      <c r="A18" s="99" t="inlineStr">
+        <is>
+          <t>Revenue recognition</t>
+        </is>
+      </c>
+      <c r="B18" s="100" t="inlineStr">
+        <is>
+          <t>The period in which revenue is recorded. Recurring revenue is recognized monthly across the service period; one-time and IRU per policy.</t>
+        </is>
+      </c>
+      <c r="C18" s="101" t="inlineStr">
+        <is>
+          <t>Convention cells + IRU method</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1">
+      <c r="A19" s="99" t="inlineStr">
+        <is>
+          <t>Effective ARPU</t>
+        </is>
+      </c>
+      <c r="B19" s="100" t="inlineStr">
+        <is>
+          <t>Actual realized recurring ARPU after the ARPU step increase, computed from the model rather than the input.</t>
+        </is>
+      </c>
+      <c r="C19" s="101" t="inlineStr">
+        <is>
+          <t>Std recurring / Avg subs</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="38" customHeight="1">
+      <c r="A20" s="99" t="inlineStr">
+        <is>
+          <t>Scenario multiplier</t>
+        </is>
+      </c>
+      <c r="B20" s="100" t="inlineStr">
+        <is>
+          <t>A factor (rows 8-10, Key Assumptions) applied to a driver (additions, churn, ARPU, DF revenue, timing) to model Conservative / Base / Aggressive outcomes.</t>
+        </is>
+      </c>
+      <c r="C20" s="101" t="inlineStr">
+        <is>
+          <t>Key Assumptions rows 8-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="38" customHeight="1">
+      <c r="A21" s="99" t="inlineStr">
+        <is>
+          <t>MTDC / F&amp;A</t>
+        </is>
+      </c>
+      <c r="B21" s="100" t="inlineStr">
+        <is>
+          <t>(Reference only) Modified Total Direct Cost / Facilities &amp; Administrative — not modeled here; revenue-only workbook.</t>
+        </is>
+      </c>
+      <c r="C21" s="101" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="38" customHeight="1">
+      <c r="A22" s="99" t="inlineStr">
+        <is>
+          <t>Expiration alert</t>
+        </is>
+      </c>
+      <c r="B22" s="100" t="inlineStr">
+        <is>
+          <t>Contract expiry flag vs 12/31/2027: RED ≤90 days, YELLOW ≤180 days, GREEN &gt;180 days, EXPIRED before year-end.</t>
+        </is>
+      </c>
+      <c r="C22" s="101" t="inlineStr">
+        <is>
+          <t>Dark Fiber Forecast status column</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="38" customHeight="1">
+      <c r="A23" s="99" t="inlineStr">
+        <is>
+          <t>Variable cost</t>
+        </is>
+      </c>
+      <c r="B23" s="100" t="inlineStr">
+        <is>
+          <t>A cost that rises and falls with revenue/volume (bandwidth, transport, commissions, payment processing). Entered as a % of revenue.</t>
+        </is>
+      </c>
+      <c r="C23" s="101" t="inlineStr">
+        <is>
+          <t>Margin Calculator B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="38" customHeight="1">
+      <c r="A24" s="99" t="inlineStr">
+        <is>
+          <t>Fixed cost</t>
+        </is>
+      </c>
+      <c r="B24" s="100" t="inlineStr">
+        <is>
+          <t>A cost that does not change with short-run revenue (network O&amp;M, salaries/G&amp;A, sales &amp; marketing, depreciation, overhead).</t>
+        </is>
+      </c>
+      <c r="C24" s="101" t="inlineStr">
+        <is>
+          <t>Margin Calculator B7:B11</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="38" customHeight="1">
+      <c r="A25" s="99" t="inlineStr">
+        <is>
+          <t>Contribution margin</t>
+        </is>
+      </c>
+      <c r="B25" s="100" t="inlineStr">
+        <is>
+          <t>Revenue minus variable costs, i.e. Revenue x (1 - variable %). The dollars left over to cover fixed costs and profit.</t>
+        </is>
+      </c>
+      <c r="C25" s="101" t="inlineStr">
+        <is>
+          <t>Margin Calculator B20 / B13</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="38" customHeight="1">
+      <c r="A26" s="99" t="inlineStr">
+        <is>
+          <t>Breakeven revenue</t>
+        </is>
+      </c>
+      <c r="B26" s="100" t="inlineStr">
+        <is>
+          <t>The revenue at which operating profit is exactly zero: Fixed costs / (1 - variable %).</t>
+        </is>
+      </c>
+      <c r="C26" s="101" t="inlineStr">
+        <is>
+          <t>Margin Calculator B24</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="38" customHeight="1">
+      <c r="A27" s="99" t="inlineStr">
+        <is>
+          <t>Operating profit (EBIT)</t>
+        </is>
+      </c>
+      <c r="B27" s="100" t="inlineStr">
+        <is>
+          <t>Pre-tax profit from operations: Revenue x (1 - variable %) - fixed costs. Excludes interest and taxes.</t>
+        </is>
+      </c>
+      <c r="C27" s="101" t="inlineStr">
+        <is>
+          <t>Margin Calculator B22</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="38" customHeight="1">
+      <c r="A28" s="99" t="inlineStr">
+        <is>
+          <t>Target-profit required revenue</t>
+        </is>
+      </c>
+      <c r="B28" s="100" t="inlineStr">
+        <is>
+          <t>Revenue needed for a chosen profit margin m: Fixed / (1 - variable % - m). For a dollar target P: (Fixed + P) / (1 - variable %).</t>
+        </is>
+      </c>
+      <c r="C28" s="101" t="inlineStr">
+        <is>
+          <t>Margin Calculator section C</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="38" customHeight="1">
+      <c r="A29" s="99" t="inlineStr">
+        <is>
+          <t>Margin of safety</t>
+        </is>
+      </c>
+      <c r="B29" s="100" t="inlineStr">
+        <is>
+          <t>How far revenue exceeds breakeven, in dollars and %. A cushion measure — larger is safer.</t>
+        </is>
+      </c>
+      <c r="C29" s="101" t="inlineStr">
+        <is>
+          <t>Margin Calculator B25:B26</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <s:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <s:sheetPr>
@@ -16012,379 +16618,813 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00808080"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>DATA DICTIONARY &amp; DEFINITIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Definitions of every major term, assumption, and calculation used in this workbook.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="47" t="inlineStr">
-        <is>
-          <t>Term / Metric</t>
-        </is>
-      </c>
-      <c r="B3" s="47" t="inlineStr">
-        <is>
-          <t>Definition</t>
-        </is>
-      </c>
-      <c r="C3" s="47" t="inlineStr">
-        <is>
-          <t>Where used / Formula</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="87" t="inlineStr">
-        <is>
-          <t>ARPU</t>
-        </is>
-      </c>
-      <c r="B4" s="88" t="inlineStr">
-        <is>
-          <t>Average Revenue Per User — recurring revenue divided by the average number of billable customers in a month.</t>
-        </is>
-      </c>
-      <c r="C4" s="89" t="inlineStr">
-        <is>
-          <t>Recurring revenue / Avg billable subs</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="87" t="inlineStr">
-        <is>
-          <t>MRR</t>
-        </is>
-      </c>
-      <c r="B5" s="88" t="inlineStr">
-        <is>
-          <t>Monthly Recurring Revenue — contractually recurring revenue in a month, excluding one-time charges (installation, activation, construction, upfront IRU).</t>
-        </is>
-      </c>
-      <c r="C5" s="89" t="inlineStr">
-        <is>
-          <t>Total recurring revenue (Consolidated)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="87" t="inlineStr">
-        <is>
-          <t>ARR run rate</t>
-        </is>
-      </c>
-      <c r="B6" s="88" t="inlineStr">
-        <is>
-          <t>Annualized Recurring Revenue — the current month's MRR multiplied by 12; a forward run-rate, not a sum of the year.</t>
-        </is>
-      </c>
-      <c r="C6" s="89" t="inlineStr">
-        <is>
-          <t>MRR x 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="87" t="inlineStr">
-        <is>
-          <t>Gross additions</t>
-        </is>
-      </c>
-      <c r="B7" s="88" t="inlineStr">
-        <is>
-          <t>New customers connected in a month before subtracting churn or disconnects.</t>
-        </is>
-      </c>
-      <c r="C7" s="89" t="inlineStr">
-        <is>
-          <t>Assumption × scenario add multiplier</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="87" t="inlineStr">
-        <is>
-          <t>Net additions</t>
-        </is>
-      </c>
-      <c r="B8" s="88" t="inlineStr">
-        <is>
-          <t>Gross additions + reconnects − churn disconnects − other disconnects.</t>
-        </is>
-      </c>
-      <c r="C8" s="89" t="inlineStr">
-        <is>
-          <t>Roll-forward</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="87" t="inlineStr">
-        <is>
-          <t>Churn</t>
-        </is>
-      </c>
-      <c r="B9" s="88" t="inlineStr">
-        <is>
-          <t>Customers who disconnect voluntarily or involuntarily. Monthly churn % is applied to the beginning subscriber base.</t>
-        </is>
-      </c>
-      <c r="C9" s="89" t="inlineStr">
-        <is>
-          <t>Beginning subs × churn % × churn multiplier</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="87" t="inlineStr">
-        <is>
-          <t>Reconnects</t>
-        </is>
-      </c>
-      <c r="B10" s="88" t="inlineStr">
-        <is>
-          <t>Previously disconnected customers who reconnect in the month; added back to the base.</t>
-        </is>
-      </c>
-      <c r="C10" s="89" t="inlineStr">
-        <is>
-          <t>Assumption input</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="38" customHeight="1">
-      <c r="A11" s="87" t="inlineStr">
-        <is>
-          <t>Average billable customers</t>
-        </is>
-      </c>
-      <c r="B11" s="88" t="inlineStr">
-        <is>
-          <t>Convention for revenue timing. 'Average' = (beginning + ending)/2; alternatives are Beginning or Ending.</t>
-        </is>
-      </c>
-      <c r="C11" s="89" t="inlineStr">
-        <is>
-          <t>Key Assumptions convention cell</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="38" customHeight="1">
-      <c r="A12" s="87" t="inlineStr">
-        <is>
-          <t>Recurring revenue</t>
-        </is>
-      </c>
-      <c r="B12" s="88" t="inlineStr">
-        <is>
-          <t>Revenue that repeats every month under a subscription or contract (broadband, DIA, static IP, managed Wi-Fi, dark fiber lease, O&amp;M).</t>
-        </is>
-      </c>
-      <c r="C12" s="89" t="inlineStr">
-        <is>
-          <t>Segment recurring rows</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="38" customHeight="1">
-      <c r="A13" s="87" t="inlineStr">
-        <is>
-          <t>One-time revenue</t>
-        </is>
-      </c>
-      <c r="B13" s="88" t="inlineStr">
-        <is>
-          <t>Non-repeating charges: installation, activation, aid-to-construction, professional services, upfront IRU proceeds.</t>
-        </is>
-      </c>
-      <c r="C13" s="89" t="inlineStr">
-        <is>
-          <t>Segment one-time rows</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="38" customHeight="1">
-      <c r="A14" s="87" t="inlineStr">
-        <is>
-          <t>IRU</t>
-        </is>
-      </c>
-      <c r="B14" s="88" t="inlineStr">
-        <is>
-          <t>Indefeasible Right of Use — a long-term (often 15-20 yr) prepaid right to use specific fiber strands. Upfront proceeds may be recognized immediately, straight-line over the term, or per a manual schedule. TREATMENT REQUIRES CFO / EXTERNAL ACCOUNTANT REVIEW UNDER ASC 606.</t>
-        </is>
-      </c>
-      <c r="C14" s="89" t="inlineStr">
-        <is>
-          <t>Dark Fiber Forecast IRU rows</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="38" customHeight="1">
-      <c r="A15" s="87" t="inlineStr">
-        <is>
-          <t>Dark fiber</t>
-        </is>
-      </c>
-      <c r="B15" s="88" t="inlineStr">
-        <is>
-          <t>Unlit optical fiber leased to a customer who provides their own optronics; billed as a monthly lease, strand/pair lease, or IRU.</t>
-        </is>
-      </c>
-      <c r="C15" s="89" t="inlineStr">
-        <is>
-          <t>Dark Fiber Forecast</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="38" customHeight="1">
-      <c r="A16" s="87" t="inlineStr">
-        <is>
-          <t>O&amp;M revenue</t>
-        </is>
-      </c>
-      <c r="B16" s="88" t="inlineStr">
-        <is>
-          <t>Operations &amp; Maintenance revenue — recurring fees for maintaining leased fiber (locates, splice repair, monitoring).</t>
-        </is>
-      </c>
-      <c r="C16" s="89" t="inlineStr">
-        <is>
-          <t>Dark Fiber Forecast O&amp;M row</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="38" customHeight="1">
-      <c r="A17" s="87" t="inlineStr">
-        <is>
-          <t>Revenue run rate</t>
-        </is>
-      </c>
-      <c r="B17" s="88" t="inlineStr">
-        <is>
-          <t>A forward-looking annualized figure derived from a single period (e.g., December MRR × 12).</t>
-        </is>
-      </c>
-      <c r="C17" s="89" t="inlineStr">
-        <is>
-          <t>ARR run rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="38" customHeight="1">
-      <c r="A18" s="87" t="inlineStr">
-        <is>
-          <t>Revenue recognition</t>
-        </is>
-      </c>
-      <c r="B18" s="88" t="inlineStr">
-        <is>
-          <t>The period in which revenue is recorded. Recurring revenue is recognized monthly across the service period; one-time and IRU per policy.</t>
-        </is>
-      </c>
-      <c r="C18" s="89" t="inlineStr">
-        <is>
-          <t>Convention cells + IRU method</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="38" customHeight="1">
-      <c r="A19" s="87" t="inlineStr">
-        <is>
-          <t>Effective ARPU</t>
-        </is>
-      </c>
-      <c r="B19" s="88" t="inlineStr">
-        <is>
-          <t>Actual realized recurring ARPU after the ARPU step increase, computed from the model rather than the input.</t>
-        </is>
-      </c>
-      <c r="C19" s="89" t="inlineStr">
-        <is>
-          <t>Std recurring / Avg subs</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="38" customHeight="1">
-      <c r="A20" s="87" t="inlineStr">
-        <is>
-          <t>Scenario multiplier</t>
-        </is>
-      </c>
-      <c r="B20" s="88" t="inlineStr">
-        <is>
-          <t>A factor (rows 8-10, Key Assumptions) applied to a driver (additions, churn, ARPU, DF revenue, timing) to model Conservative / Base / Aggressive outcomes.</t>
-        </is>
-      </c>
-      <c r="C20" s="89" t="inlineStr">
-        <is>
-          <t>Key Assumptions rows 8-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="38" customHeight="1">
-      <c r="A21" s="87" t="inlineStr">
-        <is>
-          <t>MTDC / F&amp;A</t>
-        </is>
-      </c>
-      <c r="B21" s="88" t="inlineStr">
-        <is>
-          <t>(Reference only) Modified Total Direct Cost / Facilities &amp; Administrative — not modeled here; revenue-only workbook.</t>
-        </is>
-      </c>
-      <c r="C21" s="89" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="38" customHeight="1">
-      <c r="A22" s="87" t="inlineStr">
-        <is>
-          <t>Expiration alert</t>
-        </is>
-      </c>
-      <c r="B22" s="88" t="inlineStr">
-        <is>
-          <t>Contract expiry flag vs 12/31/2027: RED ≤90 days, YELLOW ≤180 days, GREEN &gt;180 days, EXPIRED before year-end.</t>
-        </is>
-      </c>
-      <c r="C22" s="89" t="inlineStr">
-        <is>
-          <t>Dark Fiber Forecast status column</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
+<s:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <s:sheetPr>
+    <s:tabColor rgb="0070AD47"/>
+    <s:outlinePr summaryBelow="1" summaryRight="1"/>
+    <s:pageSetUpPr/>
+  </s:sheetPr>
+  <s:dimension ref="A1:G57"/>
+  <s:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <s:cols>
+    <s:col width="46" customWidth="1" min="1" max="1"/>
+    <s:col width="18" customWidth="1" min="2" max="2"/>
+    <s:col width="3" customWidth="1" min="3" max="3"/>
+    <s:col width="16" customWidth="1" min="4" max="4"/>
+    <s:col width="16" customWidth="1" min="5" max="5"/>
+    <s:col width="16" customWidth="1" min="6" max="6"/>
+    <s:col width="16" customWidth="1" min="7" max="7"/>
+  </s:cols>
+  <s:sheetData>
+    <s:row r="1" ht="30" customHeight="1">
+      <s:c r="A1" s="1" t="inlineStr">
+        <s:is>
+          <s:t>MARGIN CALCULATOR — Revenue required for a target profit</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="2">
+      <s:c r="A2" s="2" t="inlineStr">
+        <s:is>
+          <s:t>Cost-Volume-Profit (CVP) model. Enter your cost structure (blue/yellow); the calculator solves the revenue needed for any target profit. Operating profit is pre-tax (EBIT).</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="3">
+      <s:c r="F3" s="16" t="inlineStr">
+        <s:is>
+          <s:t>LEGEND</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="4">
+      <s:c r="A4" s="15" t="inlineStr">
+        <s:is>
+          <s:t>A.  COST STRUCTURE  (placeholders — replace with RIVR Tech actuals)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="F4" s="19" t="inlineStr">
+        <s:is>
+          <s:t>Editable input</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="5">
+      <s:c r="A5" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Variable operating cost (% of revenue)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B5" s="87" t="n">
+        <s:v>0.25</s:v>
+      </s:c>
+      <s:c r="C5" s="88" t="inlineStr">
+        <s:is>
+          <s:t>PLACEHOLDER</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="F5" s="22" t="inlineStr">
+        <s:is>
+          <s:t>Must-fill placeholder</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="6">
+      <s:c r="A6" s="3" t="inlineStr">
+        <s:is>
+          <s:t>Fixed operating costs (annual $):</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="F6" s="20" t="inlineStr">
+        <s:is>
+          <s:t>Calculated</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="7">
+      <s:c r="A7" s="13" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">   Network operations &amp; maintenance</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B7" s="89" t="n">
+        <s:v>2000000</s:v>
+      </s:c>
+      <s:c r="C7" s="88" t="inlineStr">
+        <s:is>
+          <s:t>PLACEHOLDER</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="8">
+      <s:c r="A8" s="13" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">   Salaries, wages &amp; benefits (G&amp;A)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B8" s="89" t="n">
+        <s:v>3500000</s:v>
+      </s:c>
+      <s:c r="C8" s="88" t="inlineStr">
+        <s:is>
+          <s:t>PLACEHOLDER</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="9">
+      <s:c r="A9" s="13" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">   Sales &amp; marketing</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B9" s="89" t="n">
+        <s:v>1200000</s:v>
+      </s:c>
+      <s:c r="C9" s="88" t="inlineStr">
+        <s:is>
+          <s:t>PLACEHOLDER</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="10">
+      <s:c r="A10" s="13" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">   Depreciation &amp; amortization</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B10" s="89" t="n">
+        <s:v>1800000</s:v>
+      </s:c>
+      <s:c r="C10" s="88" t="inlineStr">
+        <s:is>
+          <s:t>PLACEHOLDER</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="11">
+      <s:c r="A11" s="13" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">   Other overhead</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B11" s="89" t="n">
+        <s:v>500000</s:v>
+      </s:c>
+      <s:c r="C11" s="88" t="inlineStr">
+        <s:is>
+          <s:t>PLACEHOLDER</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="12">
+      <s:c r="A12" s="3" t="inlineStr">
+        <s:is>
+          <s:t>Total fixed operating costs (auto)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B12" s="90">
+        <s:f>SUM(B7:B11)</s:f>
+        <s:v>9000000</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="13">
+      <s:c r="A13" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Contribution margin % (= 1 − variable %)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B13" s="91">
+        <s:f>1-B5</s:f>
+        <s:v>0.75</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="15">
+      <s:c r="A15" s="15" t="inlineStr">
+        <s:is>
+          <s:t>B.  PROFITABILITY AT FORECAST REVENUE</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="16">
+      <s:c r="A16" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Forecast net revenue — active scenario (auto)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B16" s="92">
+        <s:f>'Consolidated Revenue'!N30</s:f>
+        <s:v>14870324.607175</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="17">
+      <s:c r="A17" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Revenue override (optional)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B17" s="34" t="n"/>
+    </s:row>
+    <s:row r="18">
+      <s:c r="A18" s="3" t="inlineStr">
+        <s:is>
+          <s:t>Revenue used</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B18" s="90">
+        <s:f>IF(B17="",B16,B17)</s:f>
+        <s:v>14870324.607175</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="19">
+      <s:c r="A19" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Variable costs</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B19" s="93">
+        <s:f>B18*B5</s:f>
+        <s:v>3717581.15179375</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="20">
+      <s:c r="A20" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Contribution margin ($)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B20" s="93">
+        <s:f>B18-B19</s:f>
+        <s:v>11152743.45538125</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="21">
+      <s:c r="A21" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Fixed operating costs</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B21" s="93">
+        <s:f>B12</s:f>
+        <s:v>9000000</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="22">
+      <s:c r="A22" s="3" t="inlineStr">
+        <s:is>
+          <s:t>Operating profit (EBIT)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B22" s="90">
+        <s:f>B20-B21</s:f>
+        <s:v>2152743.45538125</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="23">
+      <s:c r="A23" s="3" t="inlineStr">
+        <s:is>
+          <s:t>Operating profit margin %</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B23" s="94">
+        <s:f>IFERROR(B22/B18,0)</s:f>
+        <s:v>0.14476775136048756</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="24">
+      <s:c r="A24" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Breakeven revenue (profit = 0)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B24" s="93">
+        <s:f>IFERROR(B12/(1-B5),0)</s:f>
+        <s:v>12000000</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="25">
+      <s:c r="A25" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Margin of safety (revenue above breakeven)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B25" s="93">
+        <s:f>B18-B24</s:f>
+        <s:v>2870324.607175</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="26">
+      <s:c r="A26" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Margin of safety %</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B26" s="91">
+        <s:f>IFERROR(B25/B18,0)</s:f>
+        <s:v>0.19302366848065006</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="28">
+      <s:c r="A28" s="15" t="inlineStr">
+        <s:is>
+          <s:t>C.  TARGET PROFIT  →  REQUIRED REVENUE</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="29">
+      <s:c r="A29" s="17" t="inlineStr">
+        <s:is>
+          <s:t>Target profit margin (%)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B29" s="87" t="n">
+        <s:v>0.1</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="30">
+      <s:c r="A30" s="3" t="inlineStr">
+        <s:is>
+          <s:t>Required revenue for target margin</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B30" s="90">
+        <s:f>IF((1-B5-B29)&lt;=0,"Not achievable — target ≥ contribution margin",B12/(1-B5-B29))</s:f>
+        <s:v>13846153.846153846</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="31">
+      <s:c r="A31" s="13" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">   Required monthly revenue</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B31" s="93">
+        <s:f>IF(ISNUMBER(B30),B30/12,"n/a")</s:f>
+        <s:v>1153846.1538461538</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="32">
+      <s:c r="A32" s="13" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">   Resulting operating profit ($)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B32" s="93">
+        <s:f>IF(ISNUMBER(B30),B29*B30,"n/a")</s:f>
+        <s:v>1384615.3846153847</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="33">
+      <s:c r="A33" s="13" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">   Revenue vs forecast ($)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B33" s="93">
+        <s:f>IF(ISNUMBER(B30),B30-B18,"n/a")</s:f>
+        <s:v>-1024170.761021154</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="34">
+      <s:c r="A34" s="13" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">   Revenue vs forecast (%)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B34" s="91">
+        <s:f>IF(ISNUMBER(B30),IFERROR(B30/B18-1,0),"n/a")</s:f>
+        <s:v>-0.06887346363151936</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="36">
+      <s:c r="A36" s="17" t="inlineStr">
+        <s:is>
+          <s:t>Target profit — dollars ($)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B36" s="89" t="n">
+        <s:v>1500000</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="37">
+      <s:c r="A37" s="3" t="inlineStr">
+        <s:is>
+          <s:t>Required revenue for target profit $</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B37" s="90">
+        <s:f>IFERROR((B12+B36)/(1-B5),0)</s:f>
+        <s:v>14000000</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="38">
+      <s:c r="A38" s="13" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">   Revenue vs forecast ($)</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B38" s="93">
+        <s:f>B37-B18</s:f>
+        <s:v>-870324.607175</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="40">
+      <s:c r="A40" s="15" t="inlineStr">
+        <s:is>
+          <s:t>D.  TARGET-MARGIN SENSITIVITY</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="41">
+      <s:c r="A41" s="23" t="inlineStr">
+        <s:is>
+          <s:t>Target margin</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B41" s="23" t="inlineStr">
+        <s:is>
+          <s:t>Required revenue</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C41" s="23" t="inlineStr">
+        <s:is>
+          <s:t>Required monthly</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D41" s="23" t="inlineStr">
+        <s:is>
+          <s:t>Operating profit</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="E41" s="23" t="inlineStr">
+        <s:is>
+          <s:t>vs forecast rev</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="F41" s="23" t="inlineStr">
+        <s:is>
+          <s:t>Achievable?</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="42">
+      <s:c r="A42" s="33" t="n">
+        <s:v>0</s:v>
+      </s:c>
+      <s:c r="B42" s="93">
+        <s:f>IF((1-$B$5-A42)&lt;=0,"n/a",$B$12/(1-$B$5-A42))</s:f>
+        <s:v>12000000</s:v>
+      </s:c>
+      <s:c r="C42" s="93">
+        <s:f>IF(ISNUMBER(B42),B42/12,"n/a")</s:f>
+        <s:v>1000000</s:v>
+      </s:c>
+      <s:c r="D42" s="93">
+        <s:f>IF(ISNUMBER(B42),A42*B42,"n/a")</s:f>
+        <s:v>0</s:v>
+      </s:c>
+      <s:c r="E42" s="93">
+        <s:f>IF(ISNUMBER(B42),B42-$B$18,"n/a")</s:f>
+        <s:v>-2870324.607175</s:v>
+      </s:c>
+      <s:c r="F42" s="65" t="str">
+        <s:f>IF(NOT(ISNUMBER(B42)),"NO",IF(B42&lt;=$B$18,"YES — forecast covers it","Need +revenue"))</s:f>
+        <s:v>YES — forecast covers it</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="43">
+      <s:c r="A43" s="33" t="n">
+        <s:v>0.05</s:v>
+      </s:c>
+      <s:c r="B43" s="93">
+        <s:f>IF((1-$B$5-A43)&lt;=0,"n/a",$B$12/(1-$B$5-A43))</s:f>
+        <s:v>12857142.857142858</s:v>
+      </s:c>
+      <s:c r="C43" s="93">
+        <s:f>IF(ISNUMBER(B43),B43/12,"n/a")</s:f>
+        <s:v>1071428.5714285716</s:v>
+      </s:c>
+      <s:c r="D43" s="93">
+        <s:f>IF(ISNUMBER(B43),A43*B43,"n/a")</s:f>
+        <s:v>642857.142857143</s:v>
+      </s:c>
+      <s:c r="E43" s="93">
+        <s:f>IF(ISNUMBER(B43),B43-$B$18,"n/a")</s:f>
+        <s:v>-2013181.7500321418</s:v>
+      </s:c>
+      <s:c r="F43" s="65" t="str">
+        <s:f>IF(NOT(ISNUMBER(B43)),"NO",IF(B43&lt;=$B$18,"YES — forecast covers it","Need +revenue"))</s:f>
+        <s:v>YES — forecast covers it</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="44">
+      <s:c r="A44" s="33" t="n">
+        <s:v>0.1</s:v>
+      </s:c>
+      <s:c r="B44" s="93">
+        <s:f>IF((1-$B$5-A44)&lt;=0,"n/a",$B$12/(1-$B$5-A44))</s:f>
+        <s:v>13846153.846153846</s:v>
+      </s:c>
+      <s:c r="C44" s="93">
+        <s:f>IF(ISNUMBER(B44),B44/12,"n/a")</s:f>
+        <s:v>1153846.1538461538</s:v>
+      </s:c>
+      <s:c r="D44" s="93">
+        <s:f>IF(ISNUMBER(B44),A44*B44,"n/a")</s:f>
+        <s:v>1384615.3846153847</s:v>
+      </s:c>
+      <s:c r="E44" s="93">
+        <s:f>IF(ISNUMBER(B44),B44-$B$18,"n/a")</s:f>
+        <s:v>-1024170.761021154</s:v>
+      </s:c>
+      <s:c r="F44" s="65" t="str">
+        <s:f>IF(NOT(ISNUMBER(B44)),"NO",IF(B44&lt;=$B$18,"YES — forecast covers it","Need +revenue"))</s:f>
+        <s:v>YES — forecast covers it</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="45">
+      <s:c r="A45" s="33" t="n">
+        <s:v>0.15</s:v>
+      </s:c>
+      <s:c r="B45" s="93">
+        <s:f>IF((1-$B$5-A45)&lt;=0,"n/a",$B$12/(1-$B$5-A45))</s:f>
+        <s:v>15000000</s:v>
+      </s:c>
+      <s:c r="C45" s="93">
+        <s:f>IF(ISNUMBER(B45),B45/12,"n/a")</s:f>
+        <s:v>1250000</s:v>
+      </s:c>
+      <s:c r="D45" s="93">
+        <s:f>IF(ISNUMBER(B45),A45*B45,"n/a")</s:f>
+        <s:v>2250000</s:v>
+      </s:c>
+      <s:c r="E45" s="93">
+        <s:f>IF(ISNUMBER(B45),B45-$B$18,"n/a")</s:f>
+        <s:v>129675.39282499999</s:v>
+      </s:c>
+      <s:c r="F45" s="65" t="str">
+        <s:f>IF(NOT(ISNUMBER(B45)),"NO",IF(B45&lt;=$B$18,"YES — forecast covers it","Need +revenue"))</s:f>
+        <s:v>Need +revenue</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="46">
+      <s:c r="A46" s="33" t="n">
+        <s:v>0.2</s:v>
+      </s:c>
+      <s:c r="B46" s="93">
+        <s:f>IF((1-$B$5-A46)&lt;=0,"n/a",$B$12/(1-$B$5-A46))</s:f>
+        <s:v>16363636.363636361</s:v>
+      </s:c>
+      <s:c r="C46" s="93">
+        <s:f>IF(ISNUMBER(B46),B46/12,"n/a")</s:f>
+        <s:v>1363636.3636363635</s:v>
+      </s:c>
+      <s:c r="D46" s="93">
+        <s:f>IF(ISNUMBER(B46),A46*B46,"n/a")</s:f>
+        <s:v>3272727.2727272725</s:v>
+      </s:c>
+      <s:c r="E46" s="93">
+        <s:f>IF(ISNUMBER(B46),B46-$B$18,"n/a")</s:f>
+        <s:v>1493311.7564613614</s:v>
+      </s:c>
+      <s:c r="F46" s="65" t="str">
+        <s:f>IF(NOT(ISNUMBER(B46)),"NO",IF(B46&lt;=$B$18,"YES — forecast covers it","Need +revenue"))</s:f>
+        <s:v>Need +revenue</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="47">
+      <s:c r="A47" s="33" t="n">
+        <s:v>0.25</s:v>
+      </s:c>
+      <s:c r="B47" s="93">
+        <s:f>IF((1-$B$5-A47)&lt;=0,"n/a",$B$12/(1-$B$5-A47))</s:f>
+        <s:v>18000000</s:v>
+      </s:c>
+      <s:c r="C47" s="93">
+        <s:f>IF(ISNUMBER(B47),B47/12,"n/a")</s:f>
+        <s:v>1500000</s:v>
+      </s:c>
+      <s:c r="D47" s="93">
+        <s:f>IF(ISNUMBER(B47),A47*B47,"n/a")</s:f>
+        <s:v>4500000</s:v>
+      </s:c>
+      <s:c r="E47" s="93">
+        <s:f>IF(ISNUMBER(B47),B47-$B$18,"n/a")</s:f>
+        <s:v>3129675.392825</s:v>
+      </s:c>
+      <s:c r="F47" s="65" t="str">
+        <s:f>IF(NOT(ISNUMBER(B47)),"NO",IF(B47&lt;=$B$18,"YES — forecast covers it","Need +revenue"))</s:f>
+        <s:v>Need +revenue</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="48">
+      <s:c r="A48" s="33" t="n">
+        <s:v>0.3</s:v>
+      </s:c>
+      <s:c r="B48" s="93">
+        <s:f>IF((1-$B$5-A48)&lt;=0,"n/a",$B$12/(1-$B$5-A48))</s:f>
+        <s:v>20000000</s:v>
+      </s:c>
+      <s:c r="C48" s="93">
+        <s:f>IF(ISNUMBER(B48),B48/12,"n/a")</s:f>
+        <s:v>1666666.6666666667</s:v>
+      </s:c>
+      <s:c r="D48" s="93">
+        <s:f>IF(ISNUMBER(B48),A48*B48,"n/a")</s:f>
+        <s:v>6000000</s:v>
+      </s:c>
+      <s:c r="E48" s="93">
+        <s:f>IF(ISNUMBER(B48),B48-$B$18,"n/a")</s:f>
+        <s:v>5129675.392825</s:v>
+      </s:c>
+      <s:c r="F48" s="65" t="str">
+        <s:f>IF(NOT(ISNUMBER(B48)),"NO",IF(B48&lt;=$B$18,"YES — forecast covers it","Need +revenue"))</s:f>
+        <s:v>Need +revenue</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="50">
+      <s:c r="A50" s="15" t="inlineStr">
+        <s:is>
+          <s:t>E.  OPERATING MARGIN AT EACH SCENARIO'S REVENUE</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="51">
+      <s:c r="A51" s="23" t="inlineStr">
+        <s:is>
+          <s:t>Scenario</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B51" s="23" t="inlineStr">
+        <s:is>
+          <s:t>Net revenue</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C51" s="23" t="inlineStr">
+        <s:is>
+          <s:t>Operating profit</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="D51" s="23" t="inlineStr">
+        <s:is>
+          <s:t>Operating margin %</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="52">
+      <s:c r="A52" s="3" t="inlineStr">
+        <s:is>
+          <s:t>Conservative</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B52" s="95">
+        <s:f>'Scenario Analysis'!N19</s:f>
+        <s:v>13922067.325914</s:v>
+      </s:c>
+      <s:c r="C52" s="96">
+        <s:f>B52*(1-$B$5)-$B$12</s:f>
+        <s:v>1441550.4944355004</s:v>
+      </s:c>
+      <s:c r="D52" s="97">
+        <s:f>IFERROR(C52/B52,0)</s:f>
+        <s:v>0.10354428409868797</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="53">
+      <s:c r="A53" s="3" t="inlineStr">
+        <s:is>
+          <s:t>Base</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B53" s="95">
+        <s:f>'Scenario Analysis'!N35</s:f>
+        <s:v>14870324.607175</s:v>
+      </s:c>
+      <s:c r="C53" s="96">
+        <s:f>B53*(1-$B$5)-$B$12</s:f>
+        <s:v>2152743.45538125</s:v>
+      </s:c>
+      <s:c r="D53" s="97">
+        <s:f>IFERROR(C53/B53,0)</s:f>
+        <s:v>0.14476775136048756</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="54">
+      <s:c r="A54" s="3" t="inlineStr">
+        <s:is>
+          <s:t>Aggressive</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B54" s="95">
+        <s:f>'Scenario Analysis'!N51</s:f>
+        <s:v>15811838.021082252</s:v>
+      </s:c>
+      <s:c r="C54" s="96">
+        <s:f>B54*(1-$B$5)-$B$12</s:f>
+        <s:v>2858878.515811689</s:v>
+      </s:c>
+      <s:c r="D54" s="97">
+        <s:f>IFERROR(C54/B54,0)</s:f>
+        <s:v>0.18080621063787064</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="56">
+      <s:c r="A56" s="12" t="inlineStr">
+        <s:is>
+          <s:t>Model: Operating profit = Revenue × (1 − variable %) − fixed costs.  Required revenue for margin m = Fixed ÷ (1 − variable % − m).</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B56" s="69" t="n"/>
+      <s:c r="C56" s="69" t="n"/>
+      <s:c r="D56" s="69" t="n"/>
+      <s:c r="E56" s="69" t="n"/>
+      <s:c r="F56" s="69" t="n"/>
+      <s:c r="G56" s="70" t="n"/>
+    </s:row>
+    <s:row r="57">
+      <s:c r="A57" s="98" t="inlineStr">
+        <s:is>
+          <s:t>Costs are pre-tax operating costs and are PLACEHOLDERS. Replace with RIVR Tech actuals; confirm cost classification with the CFO.</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B57" s="69" t="n"/>
+      <s:c r="C57" s="69" t="n"/>
+      <s:c r="D57" s="69" t="n"/>
+      <s:c r="E57" s="69" t="n"/>
+      <s:c r="F57" s="69" t="n"/>
+      <s:c r="G57" s="70" t="n"/>
+    </s:row>
+  </s:sheetData>
+  <s:mergeCells count="9">
+    <s:mergeCell ref="A4:B4"/>
+    <s:mergeCell ref="A1:G1"/>
+    <s:mergeCell ref="A15:B15"/>
+    <s:mergeCell ref="A56:G56"/>
+    <s:mergeCell ref="A50:D50"/>
+    <s:mergeCell ref="A28:B28"/>
+    <s:mergeCell ref="A2:G2"/>
+    <s:mergeCell ref="A40:F40"/>
+    <s:mergeCell ref="A57:G57"/>
+  </s:mergeCells>
+  <s:conditionalFormatting sqref="B22">
+    <s:cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="6">
+      <s:formula>0</s:formula>
+    </s:cfRule>
+    <s:cfRule type="cellIs" priority="2" operator="lessThan" dxfId="7">
+      <s:formula>0</s:formula>
+    </s:cfRule>
+  </s:conditionalFormatting>
+  <s:conditionalFormatting sqref="B23">
+    <s:cfRule type="cellIs" priority="3" operator="lessThan" dxfId="7">
+      <s:formula>0</s:formula>
+    </s:cfRule>
+  </s:conditionalFormatting>
+  <s:conditionalFormatting sqref="E42:E48">
+    <s:cfRule type="cellIs" priority="4" operator="lessThanOrEqual" dxfId="8">
+      <s:formula>0</s:formula>
+    </s:cfRule>
+    <s:cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="9">
+      <s:formula>0</s:formula>
+    </s:cfRule>
+  </s:conditionalFormatting>
+  <s:conditionalFormatting sqref="F42:F48">
+    <s:cfRule type="expression" priority="6" dxfId="2">
+      <s:formula>ISNUMBER(SEARCH("YES",F42))</s:formula>
+    </s:cfRule>
+    <s:cfRule type="expression" priority="7" dxfId="1">
+      <s:formula>ISNUMBER(SEARCH("Need",F42))</s:formula>
+    </s:cfRule>
+  </s:conditionalFormatting>
+  <s:conditionalFormatting sqref="C52">
+    <s:cfRule type="cellIs" priority="8" operator="lessThan" dxfId="10">
+      <s:formula>0</s:formula>
+    </s:cfRule>
+  </s:conditionalFormatting>
+  <s:conditionalFormatting sqref="D52">
+    <s:cfRule type="cellIs" priority="9" operator="lessThan" dxfId="10">
+      <s:formula>0</s:formula>
+    </s:cfRule>
+  </s:conditionalFormatting>
+  <s:conditionalFormatting sqref="C53">
+    <s:cfRule type="cellIs" priority="10" operator="lessThan" dxfId="10">
+      <s:formula>0</s:formula>
+    </s:cfRule>
+  </s:conditionalFormatting>
+  <s:conditionalFormatting sqref="D53">
+    <s:cfRule type="cellIs" priority="11" operator="lessThan" dxfId="10">
+      <s:formula>0</s:formula>
+    </s:cfRule>
+  </s:conditionalFormatting>
+  <s:conditionalFormatting sqref="C54">
+    <s:cfRule type="cellIs" priority="12" operator="lessThan" dxfId="10">
+      <s:formula>0</s:formula>
+    </s:cfRule>
+  </s:conditionalFormatting>
+  <s:conditionalFormatting sqref="D54">
+    <s:cfRule type="cellIs" priority="13" operator="lessThan" dxfId="10">
+      <s:formula>0</s:formula>
+    </s:cfRule>
+  </s:conditionalFormatting>
+  <s:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <s:legacyDrawing r:id="anysvml"/>
+</s:worksheet>
 </file>
</xml_diff>